<commit_message>
Version Wed 03/11/2026 14:43:17.53
</commit_message>
<xml_diff>
--- a/Sentry/sentry_errors.xlsx
+++ b/Sentry/sentry_errors.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sales" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sales'!$A$1:$L$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sales'!$A$1:$L$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -529,17 +529,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>7294095442</t>
+          <t>7284965351</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IntegrityError: (sqlalchemy.dialects.postgresql.asyncpg.IntegrityError) &lt;class 'asyncpg.exceptions.ForeignKeyViolationError'&gt;: update or delete on table "operation_types" violates foreign key constraint "operation_config_operation_type_code_fkey" on table "operation_co...</t>
+          <t>[SEND ERROR] Traceback: Traceback (most recent call last):</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>ForeignKeyViolationError</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -548,28 +548,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>asyncpg/protocol/protocol.pyx:205</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>bind_execute</t>
-        </is>
-      </c>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
@@ -577,24 +569,24 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Исправлено удаление типа операции: добавлена корректная обработка связанных данных и возврат понятной ошибки без падения API (FK violation handled).</t>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7294095442/</t>
+          <t>https://zakharenkov.sentry.io/issues/7284965351/</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>7275717149</t>
+          <t>7278462695</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Database session error: (sqlalchemy.dialects.postgresql.asyncpg.IntegrityError) &lt;class 'asyncpg.exceptions.ForeignKeyViolationError'&gt;: update or delete on table "operation_types" violates foreign key constraint "operation_config_operation_type_code_fkey...</t>
+          <t>[SEND ERROR] Unexpected error: 'CallbackQuery' object has no attribute 'reply_text'</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -608,16 +600,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>125</v>
+        <v>1</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -629,24 +621,24 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Убрано ложное логирование 401 как database session error: HTTPException обрабатывается отдельно без записи в Sentry как ошибка БД.</t>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7275717149/</t>
+          <t>https://zakharenkov.sentry.io/issues/7278462695/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7294021913</t>
+          <t>7323450449</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ProgrammingError: (sqlalchemy.dialects.postgresql.asyncpg.ProgrammingError) &lt;class 'asyncpg.exceptions.UndefinedColumnError'&gt;: column ot.executor_role does not exist</t>
+          <t>ProgrammingError: (sqlalchemy.dialects.postgresql.asyncpg.ProgrammingError) &lt;class 'asyncpg.exceptions.UndefinedColumnError'&gt;: column "language_code" does not exist</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -660,16 +652,16 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-02-26</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -689,29 +681,29 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Исправлена совместимость со схемой БД без колонки executor_role: добавлена проверка наличия колонки и fallback-запросы для operation types.</t>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7294021913/</t>
+          <t>https://zakharenkov.sentry.io/issues/7323450449/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7278663445</t>
+          <t>7299667604</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AttributeError: 'str' object has no attribute 'get'</t>
+          <t>NetworkError: Bad Gateway</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AttributeError</t>
+          <t>NetworkError</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -720,26 +712,26 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>src/telegram_bot/handlers_expeditor.py:929</t>
+          <t>telegram/request/_baserequest.py:387</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>cb_exp_received_payments</t>
+          <t>_request_wrapper</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -754,24 +746,24 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7278663445/</t>
+          <t>https://zakharenkov.sentry.io/issues/7299667604/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7278663074</t>
+          <t>7294095442</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AttributeError: 'str' object has no attribute 'get'</t>
+          <t>IntegrityError: (sqlalchemy.dialects.postgresql.asyncpg.IntegrityError) &lt;class 'asyncpg.exceptions.ForeignKeyViolationError'&gt;: update or delete on table "operation_types" violates foreign key constraint "operation_config_operation_type_code_fkey" on table "operation_co...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AttributeError</t>
+          <t>ForeignKeyViolationError</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -780,26 +772,26 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>src/telegram_bot/handlers_expeditor.py:104</t>
+          <t>asyncpg/protocol/protocol.pyx:205</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>_get_paid_order_ids</t>
+          <t>bind_execute</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -809,29 +801,29 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+          <t>Исправлено удаление типа операции: добавлена корректная обработка связанных данных и возврат понятной ошибки без падения API (FK violation handled).</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7278663074/</t>
+          <t>https://zakharenkov.sentry.io/issues/7294095442/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7287515728</t>
+          <t>7275717149</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BadRequest: Message is not modified: specified new message content and reply markup are exactly the same as a current content and reply markup of the message</t>
+          <t>Database session error: (sqlalchemy.dialects.postgresql.asyncpg.IntegrityError) &lt;class 'asyncpg.exceptions.ForeignKeyViolationError'&gt;: update or delete on table "operation_types" violates foreign key constraint "operation_config_operation_type_code_fkey...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BadRequest</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -840,28 +832,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-19</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>telegram/request/_baserequest.py:383</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>_request_wrapper</t>
-        </is>
-      </c>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
@@ -869,29 +853,29 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+          <t>Убрано ложное логирование 401 как database session error: HTTPException обрабатывается отдельно без записи в Sentry как ошибка БД.</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7287515728/</t>
+          <t>https://zakharenkov.sentry.io/issues/7275717149/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>7279725195</t>
+          <t>7294021913</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Traceback (most recent call last):</t>
+          <t>ProgrammingError: (sqlalchemy.dialects.postgresql.asyncpg.ProgrammingError) &lt;class 'asyncpg.exceptions.UndefinedColumnError'&gt;: column ot.executor_role does not exist</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>UndefinedColumnError</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -900,20 +884,28 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-26</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>asyncpg/protocol/protocol.pyx:165</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>prepare</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
@@ -921,29 +913,29 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+          <t>Исправлена совместимость со схемой БД без колонки executor_role: добавлена проверка наличия колонки и fallback-запросы для operation types.</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7279725195/</t>
+          <t>https://zakharenkov.sentry.io/issues/7294021913/</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7278760989</t>
+          <t>7278663445</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RuntimeError: Database connection failed</t>
+          <t>AttributeError: 'str' object has no attribute 'get'</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>RuntimeError</t>
+          <t>AttributeError</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -952,7 +944,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -961,17 +953,17 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>src/main.py:62</t>
+          <t>src/telegram_bot/handlers_expeditor.py:929</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>lifespan</t>
+          <t>cb_exp_received_payments</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -986,24 +978,24 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7278760989/</t>
+          <t>https://zakharenkov.sentry.io/issues/7278663445/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>7278760957</t>
+          <t>7278663074</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Application startup failed. Exiting.</t>
+          <t>AttributeError: 'str' object has no attribute 'get'</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>AttributeError</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1012,7 +1004,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1021,11 +1013,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>src/telegram_bot/handlers_expeditor.py:104</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>_get_paid_order_ids</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
@@ -1038,24 +1038,24 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7278760957/</t>
+          <t>https://zakharenkov.sentry.io/issues/7278663074/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>7278760963</t>
+          <t>7287515728</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Database connection failed: [Errno 111] Connection refused</t>
+          <t>BadRequest: Message is not modified: specified new message content and reply markup are exactly the same as a current content and reply markup of the message</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>BadRequest</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1064,20 +1064,28 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>telegram/request/_baserequest.py:383</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>_request_wrapper</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
@@ -1090,114 +1098,330 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>https://zakharenkov.sentry.io/issues/7278760963/</t>
+          <t>https://zakharenkov.sentry.io/issues/7287515728/</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>7279725195</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Traceback (most recent call last):</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>https://zakharenkov.sentry.io/issues/7279725195/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>7278760989</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>RuntimeError: Database connection failed</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>RuntimeError</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>src/main.py:62</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>lifespan</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>https://zakharenkov.sentry.io/issues/7278760989/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>7278760957</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Application startup failed. Exiting.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>https://zakharenkov.sentry.io/issues/7278760957/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>7278760963</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Database connection failed: [Errno 111] Connection refused</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>https://zakharenkov.sentry.io/issues/7278760963/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>7279797572</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>ConnectionRefusedError: [Errno 111] Connect call failed ('45.141.76.83', 5433)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>ConnectionRefusedError</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>error</t>
         </is>
       </c>
-      <c r="E12" t="n">
+      <c r="E16" t="n">
         <v>6</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>2026-02-20</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>2026-02-23</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>asyncio/selector_events.py:691</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>_sock_connect_cb</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>RESOLVED</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Исправлено в проекте, задача закрыта и синхронизирована в Sentry.</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>https://zakharenkov.sentry.io/issues/7279797572/</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Всего ошибок в проекте:</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="B18" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Кол-во исправленных:</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="B19" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Кол-во неисправленных:</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B20" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Процент готовности:</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L12"/>
+  <autoFilter ref="A1:L16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
@@ -1210,6 +1434,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>